<commit_message>
Ajout de date_debut et date_fin dans la table collecte_instrument - Script d'intégration des tables - Fichiers de métadonnées
</commit_message>
<xml_diff>
--- a/Base_de_donnees/Fichiers_metadonnees/Metadonnees_personnes.xlsx
+++ b/Base_de_donnees/Fichiers_metadonnees/Metadonnees_personnes.xlsx
@@ -108,10 +108,10 @@
     <t xml:space="preserve">Referent/Collecteur  (R/C)</t>
   </si>
   <si>
-    <t xml:space="preserve">date_debut (si R)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">date_fin (si R)</t>
+    <t xml:space="preserve">date_debut</t>
+  </si>
+  <si>
+    <t xml:space="preserve">date_fin</t>
   </si>
   <si>
     <t xml:space="preserve">HOBO_n°02</t>
@@ -257,7 +257,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yy"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -300,12 +300,6 @@
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="0"/>
     </font>
   </fonts>
   <fills count="2">
@@ -350,7 +344,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -376,10 +370,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1801,7 +1791,7 @@
       <c r="A81" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B81" s="7" t="s">
+      <c r="B81" s="5" t="s">
         <v>70</v>
       </c>
       <c r="C81" s="1" t="s">
@@ -1815,7 +1805,7 @@
       <c r="A82" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B82" s="7" t="s">
+      <c r="B82" s="5" t="s">
         <v>70</v>
       </c>
       <c r="C82" s="1" t="s">
@@ -1827,7 +1817,7 @@
       <c r="A83" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B83" s="7" t="s">
+      <c r="B83" s="5" t="s">
         <v>71</v>
       </c>
       <c r="C83" s="1" t="s">
@@ -1841,7 +1831,7 @@
       <c r="A84" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B84" s="7" t="s">
+      <c r="B84" s="5" t="s">
         <v>71</v>
       </c>
       <c r="C84" s="1" t="s">

</xml_diff>